<commit_message>
added sql-scripts for update and delete, added images for documentation, finalized Arbeitsjournal
</commit_message>
<xml_diff>
--- a/Dokumentation/Projektplanung&Arbeitsübersicht/Arbeitsjournal.xlsx
+++ b/Dokumentation/Projektplanung&Arbeitsübersicht/Arbeitsjournal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluz-my.sharepoint.com/personal/benjamin_maier_sluz_ch/Documents/BBZW_2/Sem_2/IPT61/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluz-my.sharepoint.com/personal/benjamin_maier_sluz_ch/Documents/BBZW_2/Sem_2/IPT61/ipt-6.1_expensemanager/Dokumentation/Projektplanung&amp;Arbeitsübersicht/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{78FC798B-B897-407B-8A3F-652FB2139CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EC1986A-FD41-4F24-A720-93A7A905FBE5}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="8_{78FC798B-B897-407B-8A3F-652FB2139CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF78BC07-D203-488B-832C-5E2082BB5349}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="64">
   <si>
     <r>
       <rPr>
@@ -208,6 +208,54 @@
   </si>
   <si>
     <t xml:space="preserve">Janik: 50%, Benjamin: 50%, Hilfe von Luis für Janik </t>
+  </si>
+  <si>
+    <t>ER-Diagram, UML, Klassen und Datentypen Diagramm fertiggestellen, Arbeitsjournal nachtragen, Besprechung, Singleton Pattern, UserView erarbeiten</t>
+  </si>
+  <si>
+    <t>Skeleton für singleton-connection, UI weiterarbeit, Sigleton Pattern in homeview function erarbeitet, Dokumentation: Ablaufdiagramm erneuert, Arbeitsjournal planen</t>
+  </si>
+  <si>
+    <t>Skeleton für singleton-connection anfangen, Ablaufdiagramm anpassen, Arbeitsjournal planen</t>
+  </si>
+  <si>
+    <t>Readme überarbeiten,  Bedienungsanleitung anfangen, Display-variables für Datenbankinformationen einfügen.</t>
+  </si>
+  <si>
+    <t>Readme überarbeitet, Bedienungsanleitung angefangen, Displayvariabeln für Datenbankinformationen einfügen</t>
+  </si>
+  <si>
+    <t>ER und Relationen-Diagramm überarbeiten, Readme überarbeiten, Pflichtfelder einfügen</t>
+  </si>
+  <si>
+    <t>ER und Relationen-Diagramm überarbeitet, Readme überarbeitet, Pflichtfelder eingefügt</t>
+  </si>
+  <si>
+    <t>Bedienungsanleitung weiterarbeiten</t>
+  </si>
+  <si>
+    <t>Bedienungsanleitung weitererarbeitet, Bugfixxing</t>
+  </si>
+  <si>
+    <t>Arbeitsjournal hinzugefügen, Dokumentation anfangen (template für Inhalte erstellen)</t>
+  </si>
+  <si>
+    <t>Arbeitsjournal hinzugefügt, Dokumentation angefangen (Template für Inhalte erstellt)</t>
+  </si>
+  <si>
+    <t>Weiterarbeit Dokumentation, Aufräumen in Ordnerstruktur, Bugfixxing für singleton-verbindung</t>
+  </si>
+  <si>
+    <t>Dokumentation weiterarbeiten, Ordnerstruktur aufgeräumt, Bugfixxing für sigleton-verbindung</t>
+  </si>
+  <si>
+    <t>Singleton-Verbindung fertigstellen, Videoaufnahmen, Dokumentation überprüfen, Video aufnehmen</t>
+  </si>
+  <si>
+    <t>Projektabgabe überprüfen</t>
+  </si>
+  <si>
+    <t>Projektabgabe überprüft</t>
   </si>
 </sst>
 </file>
@@ -340,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -460,9 +508,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1969,7 +2014,7 @@
       <c r="G18" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="H18" s="40"/>
+      <c r="H18" s="18"/>
       <c r="I18" s="33"/>
       <c r="J18" s="34"/>
       <c r="K18" s="34"/>
@@ -2134,7 +2179,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="18" t="s">
@@ -2160,7 +2205,7 @@
       <c r="W23" s="34"/>
       <c r="X23" s="34"/>
     </row>
-    <row r="24" spans="1:59" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:59" ht="45" x14ac:dyDescent="0.15">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -2173,9 +2218,13 @@
       <c r="D24" s="3">
         <v>2</v>
       </c>
-      <c r="E24" s="18"/>
+      <c r="E24" s="18" t="s">
+        <v>50</v>
+      </c>
       <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
+      <c r="G24" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="H24" s="38" t="s">
         <v>46</v>
       </c>
@@ -2196,7 +2245,7 @@
       <c r="W24" s="34"/>
       <c r="X24" s="34"/>
     </row>
-    <row r="25" spans="1:59" ht="11.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:59" ht="36" x14ac:dyDescent="0.15">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -2209,9 +2258,13 @@
       <c r="D25" s="3">
         <v>2</v>
       </c>
-      <c r="E25" s="18"/>
+      <c r="E25" s="18" t="s">
+        <v>51</v>
+      </c>
       <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
+      <c r="G25" s="18" t="s">
+        <v>52</v>
+      </c>
       <c r="H25" s="38" t="s">
         <v>46</v>
       </c>
@@ -2232,7 +2285,7 @@
       <c r="W25" s="34"/>
       <c r="X25" s="34"/>
     </row>
-    <row r="26" spans="1:59" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:59" ht="27" x14ac:dyDescent="0.15">
       <c r="A26" s="3">
         <v>16</v>
       </c>
@@ -2245,9 +2298,13 @@
       <c r="D26" s="3">
         <v>2</v>
       </c>
-      <c r="E26" s="18"/>
+      <c r="E26" s="18" t="s">
+        <v>53</v>
+      </c>
       <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
+      <c r="G26" s="18" t="s">
+        <v>54</v>
+      </c>
       <c r="H26" s="38" t="s">
         <v>46</v>
       </c>
@@ -2345,9 +2402,13 @@
       <c r="D29" s="3">
         <v>2</v>
       </c>
-      <c r="E29" s="18"/>
+      <c r="E29" s="18" t="s">
+        <v>55</v>
+      </c>
       <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
+      <c r="G29" s="18" t="s">
+        <v>56</v>
+      </c>
       <c r="H29" s="38" t="s">
         <v>46</v>
       </c>
@@ -2368,7 +2429,7 @@
       <c r="W29" s="34"/>
       <c r="X29" s="34"/>
     </row>
-    <row r="30" spans="1:59" ht="18" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:59" ht="27" x14ac:dyDescent="0.15">
       <c r="A30" s="3">
         <v>20</v>
       </c>
@@ -2381,9 +2442,13 @@
       <c r="D30" s="3">
         <v>2</v>
       </c>
-      <c r="E30" s="18"/>
+      <c r="E30" s="18" t="s">
+        <v>57</v>
+      </c>
       <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
+      <c r="G30" s="18" t="s">
+        <v>58</v>
+      </c>
       <c r="H30" s="38" t="s">
         <v>46</v>
       </c>
@@ -2404,7 +2469,7 @@
       <c r="W30" s="34"/>
       <c r="X30" s="34"/>
     </row>
-    <row r="31" spans="1:59" ht="18" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:59" ht="27" x14ac:dyDescent="0.15">
       <c r="A31" s="3">
         <v>21</v>
       </c>
@@ -2417,9 +2482,13 @@
       <c r="D31" s="3">
         <v>2</v>
       </c>
-      <c r="E31" s="18"/>
+      <c r="E31" s="18" t="s">
+        <v>59</v>
+      </c>
       <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
+      <c r="G31" s="18" t="s">
+        <v>60</v>
+      </c>
       <c r="H31" s="38" t="s">
         <v>46</v>
       </c>
@@ -2440,7 +2509,7 @@
       <c r="W31" s="34"/>
       <c r="X31" s="34"/>
     </row>
-    <row r="32" spans="1:59" ht="18" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:59" ht="27" x14ac:dyDescent="0.15">
       <c r="A32" s="3">
         <v>22</v>
       </c>
@@ -2453,9 +2522,13 @@
       <c r="D32" s="3">
         <v>2</v>
       </c>
-      <c r="E32" s="18"/>
+      <c r="E32" s="18" t="s">
+        <v>61</v>
+      </c>
       <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
+      <c r="G32" s="18" t="s">
+        <v>61</v>
+      </c>
       <c r="H32" s="38" t="s">
         <v>46</v>
       </c>
@@ -2489,12 +2562,16 @@
       <c r="D33" s="3">
         <v>2</v>
       </c>
-      <c r="E33" s="12"/>
+      <c r="E33" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="F33" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G33" s="18"/>
-      <c r="H33" s="40"/>
+      <c r="G33" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H33" s="18"/>
       <c r="I33" s="33"/>
       <c r="J33" s="34"/>
       <c r="K33" s="34"/>
@@ -2564,7 +2641,7 @@
         <v>9</v>
       </c>
       <c r="G35" s="18"/>
-      <c r="H35" s="40"/>
+      <c r="H35" s="18"/>
       <c r="I35" s="33"/>
       <c r="J35" s="34"/>
       <c r="K35" s="34"/>

</xml_diff>